<commit_message>
Added today's data at 10:50 pm 26-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1308,24 +1308,38 @@
       <c r="C13" s="14">
         <v>120</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
+      <c r="D13" s="14">
+        <v>60</v>
+      </c>
+      <c r="E13" s="14">
+        <v>0</v>
+      </c>
       <c r="F13" s="14">
         <v>350</v>
       </c>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
+      <c r="G13" s="14">
+        <v>7</v>
+      </c>
+      <c r="H13" s="14">
+        <v>180</v>
+      </c>
       <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v>800</v>
+        <v>1040</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v>640</v>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 9:55 pm 27-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1343,25 +1343,47 @@
       <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B14" s="14">
+        <v>330</v>
+      </c>
+      <c r="C14" s="14">
+        <v>120</v>
+      </c>
+      <c r="D14" s="14">
+        <v>180</v>
+      </c>
+      <c r="E14" s="14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="14">
+        <v>200</v>
+      </c>
+      <c r="G14" s="14">
+        <v>4</v>
+      </c>
+      <c r="H14" s="14">
+        <v>60</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
+        <v>550</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 9:50 pm 28-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1387,25 +1387,47 @@
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B15" s="14">
+        <v>300</v>
+      </c>
+      <c r="C15" s="14">
+        <v>120</v>
+      </c>
+      <c r="D15" s="14">
+        <v>60</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>250</v>
+      </c>
+      <c r="G15" s="14">
+        <v>5</v>
+      </c>
+      <c r="H15" s="14">
+        <v>120</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+        <v>590</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 11:25 PM 29-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -213,6 +213,18 @@
   </si>
   <si>
     <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Had a great day today !</t>
   </si>
 </sst>
 </file>
@@ -1431,26 +1443,50 @@
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B16" s="14">
+        <v>480</v>
+      </c>
+      <c r="C16" s="14">
+        <v>120</v>
+      </c>
+      <c r="D16" s="14">
+        <v>390</v>
+      </c>
+      <c r="E16" s="14">
+        <v>120</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>120</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1230</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>210</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:44 PM 30-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Had a great day today !</t>
+  </si>
+  <si>
+    <t>Prepared for the CA and roam around to the campus</t>
   </si>
 </sst>
 </file>
@@ -1488,27 +1491,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B17" s="14">
+        <v>390</v>
+      </c>
+      <c r="C17" s="14">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>220</v>
+      </c>
+      <c r="E17" s="14">
+        <v>60</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>180</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>590</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>

</xml_diff>

<commit_message>
Updated today at 10:32 PM 31-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -228,6 +228,9 @@
   </si>
   <si>
     <t>Prepared for the CA and roam around to the campus</t>
+  </si>
+  <si>
+    <t>Went for a workshop of AI and had fun with friends.</t>
   </si>
 </sst>
 </file>
@@ -1537,27 +1540,51 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B18" s="14">
+        <v>390</v>
+      </c>
+      <c r="C18" s="14">
+        <v>120</v>
+      </c>
+      <c r="D18" s="14">
+        <v>120</v>
+      </c>
+      <c r="E18" s="14">
+        <v>0</v>
+      </c>
+      <c r="F18" s="14">
+        <v>150</v>
+      </c>
+      <c r="G18" s="14">
+        <v>3</v>
+      </c>
+      <c r="H18" s="14">
+        <v>240</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>

</xml_diff>

<commit_message>
Updated today at 11:38 PM 02-Sep
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -231,6 +231,12 @@
   </si>
   <si>
     <t>Went for a workshop of AI and had fun with friends.</t>
+  </si>
+  <si>
+    <t>Felt tired after classes</t>
+  </si>
+  <si>
+    <t>Felt tired after classes and had talked with new friends</t>
   </si>
 </sst>
 </file>
@@ -1587,48 +1593,96 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B19" s="14">
+        <v>450</v>
+      </c>
+      <c r="C19" s="14">
+        <v>120</v>
+      </c>
+      <c r="D19" s="14">
+        <v>120</v>
+      </c>
+      <c r="E19" s="14">
+        <v>60</v>
+      </c>
+      <c r="F19" s="14">
+        <v>350</v>
+      </c>
+      <c r="G19" s="14">
+        <v>7</v>
+      </c>
+      <c r="H19" s="14">
+        <v>120</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+        <v>220</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B20" s="14">
+        <v>390</v>
+      </c>
+      <c r="C20" s="14">
+        <v>120</v>
+      </c>
+      <c r="D20" s="14">
+        <v>120</v>
+      </c>
+      <c r="E20" s="14">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14">
+        <v>350</v>
+      </c>
+      <c r="G20" s="14">
+        <v>7</v>
+      </c>
+      <c r="H20" s="14">
+        <v>120</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>340</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>

</xml_diff>

<commit_message>
Updated today at 10:39 PM 03-Sep
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1685,25 +1685,47 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B21" s="14">
+        <v>390</v>
+      </c>
+      <c r="C21" s="14">
+        <v>0</v>
+      </c>
+      <c r="D21" s="14">
+        <v>180</v>
+      </c>
+      <c r="E21" s="14">
+        <v>60</v>
+      </c>
+      <c r="F21" s="14">
+        <v>200</v>
+      </c>
+      <c r="G21" s="14">
+        <v>4</v>
+      </c>
+      <c r="H21" s="14">
+        <v>120</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:10 PM 04-Sep
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1729,25 +1729,47 @@
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B22" s="14">
+        <v>330</v>
+      </c>
+      <c r="C22" s="14">
+        <v>120</v>
+      </c>
+      <c r="D22" s="14">
+        <v>120</v>
+      </c>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14">
+        <v>300</v>
+      </c>
+      <c r="G22" s="14">
+        <v>6</v>
+      </c>
+      <c r="H22" s="14">
+        <v>120</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
+        <v>450</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Updated today at 10:45 PM 05-Aug
</commit_message>
<xml_diff>
--- a/12604355.xlsx
+++ b/12604355.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1773,25 +1773,47 @@
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B23" s="14">
+        <v>450</v>
+      </c>
+      <c r="C23" s="14">
+        <v>120</v>
+      </c>
+      <c r="D23" s="14">
+        <v>390</v>
+      </c>
+      <c r="E23" s="14">
+        <v>120</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14">
+        <v>0</v>
+      </c>
+      <c r="H23" s="14">
+        <v>240</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1320</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
+        <v>120</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>